<commit_message>
Fill Zerde AI-idioms project with the student's experiment results
Rewrites the paper around the collected data (ChatGPT, DeepSeek,
Gemini; 182 answers): results, discussion, conclusions, annotation,
example table and full answer tables in appendix B. Research diary,
supervisor review, AI declaration and ethics sheet now reflect the
actual work. The workbook is rebuilt from the student's file with
charts; corrections are recorded in tuzetuler.json.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWp2V469ega9rMmDw4DHEN
</commit_message>
<xml_diff>
--- a/Zerde_ZhI_frazeologizm/Tazhiribe_kestesi.xlsx
+++ b/Zerde_ZhI_frazeologizm/Tazhiribe_kestesi.xlsx
@@ -1323,14 +1323,32 @@
           <t>қатты қуану</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="7" t="n"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>қатты қуану, мәз болып күлу деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G2" s="7" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="7" t="n"/>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>адамның өте қуанышты, мәз-мейрам болған күйін, яғни қатты күлуін, қуаныштан аузы құлағына жеткендей болуын білдіреді.</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J2" s="7" t="n"/>
-      <c r="K2" s="6" t="n"/>
-      <c r="L2" s="7" t="n"/>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Бұл тұрақты тіркес адамның қатты қуанғанын, мәз болып, шаттанғанын білдіреді (адам қатты күлгенде немесе жымиғанда аузының езуі кең созылатынына негізделген).</t>
+        </is>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M2" s="7" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1">
@@ -1352,14 +1370,32 @@
           <t>өкінді</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="7" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>қатты өкінді деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G3" s="7" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="7" t="n"/>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>адамның қатты өкінгенін, амалсыздан қынжылғанын, я болмаса бір нәрсеге таңырқап, таңдай қаққанын білдіреді. Көбінесе өкініш, өшпенділік немесе қызығушылық мәнінде қолданылады.</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J3" s="7" t="n"/>
-      <c r="K3" s="6" t="n"/>
-      <c r="L3" s="7" t="n"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Бұл тұрақты тіркес жіберіп алған мүмкіндікке немесе жасаған қателігіне қатты өкінуді, өкініш білдіруді білдіреді.</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M3" s="7" t="n"/>
     </row>
     <row r="4" ht="45" customHeight="1">
@@ -1381,14 +1417,32 @@
           <t>өте тез</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="7" t="n"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>өте тез, қас қағым сәтте деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G4" s="7" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="7" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>тіркес өте қысқа уақытты, лезде, тез болғандықты білдіреді. Яғни бір нәрсенің көз ашып-жұмған аралығындай жылдам жүзеге асқанын сипаттайды.</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J4" s="7" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="7" t="n"/>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>іс-әрекеттің өте жылдам, лезде, қас-қағым сәтте орын алғанын білдіреді.</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M4" s="7" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1">
@@ -1410,14 +1464,32 @@
           <t>үндемеу, сөйлемеу</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="n"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>үндемеу, ештеңе айтпау деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G5" s="7" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="7" t="n"/>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>үндемеу, ешнәрсе айтпау, сыр бермеу деген мағынаны білдіреді. Адамның тапжылмай үнсіз қалуын, тіс жарып сөйлемеуін сипаттайды.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J5" s="7" t="n"/>
-      <c r="K5" s="6" t="n"/>
-      <c r="L5" s="7" t="n"/>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>ештеңе айтпауды, мүлдем үндемеуді, тіс жармауды немесе сырды берік сақтауды білдіреді.</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M5" s="7" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1">
@@ -1439,14 +1511,32 @@
           <t>мұқият тыңдау, назар салу</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>зейін қойып, мұқият тыңдау деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G6" s="7" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="7" t="n"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>бір нәрсеге қатты назар аудару, мұқият тыңдау, сақ болу деген мағынаны білдіреді. Көбінесе «құлақ түру» түрінде де қолданылады.</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="7" t="n"/>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>бірдеңені мұқият, зейін қойып тыңдауды немесе қандай да бір жаңалықты, хабарды күтіп елеңдеуді білдіреді.</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M6" s="7" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -1468,14 +1558,32 @@
           <t>ұйықтамау</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>ұйықтамау, көз ілмеу деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G7" s="7" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="7" t="n"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>ұйықтамау, көз ілмеу, түні бойы ояу болу деген мағынаны білдіреді. Сондай-ақ бір нәрсеге қатты көңіл бөліп, көз алмай қарау мәнінде де қолданылады.</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J7" s="7" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="7" t="n"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>мүлдем ұйықтамауды, көз ілмеуді немесе бір нәрсеге өте мұқият, тапжылмай назар аударуды білдіреді (көбіне түні бойы ұйықтамай шығу мағынасында қолданылады).</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M7" s="7" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1">
@@ -1497,14 +1605,32 @@
           <t>қатты толқыды, қорықты</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="7" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>қатты қорықты, шошыды деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G8" s="7" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="7" t="n"/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>қатты қорыққанда, үрейленгенде немесе қатты толқығанда жүректің соғуы жиілеп, дүрсілдеп кетуін білдіреді. Яғни адамның қорқыныш немесе қобалжу күйін сипаттайды.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J8" s="7" t="n"/>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="7" t="n"/>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>кенеттен қатты қорқуды, үрейленуді, зәресі ұшуды білдіреді.</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M8" s="7" t="n"/>
     </row>
     <row r="9" ht="45" customHeight="1">
@@ -1526,15 +1652,41 @@
           <t>келісті</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="n"/>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>келіскенін, мақұлдағанын білдірді деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G9" s="7" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>келісім білдіру, мақұлдау, «иә» деп жауап беру деген мағынаны білдіреді. Сондай-ақ біреуге бағыныштылық, мойынсұну мәнінде де қолданылады.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>келісуді, мақұлдауды, рұқсат беруді немесе үнсіз амандасу белгісін білдіреді.</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -1555,14 +1707,32 @@
           <t>жомарт</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>жомарт, барын өзгелерден аямайтын деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G10" s="7" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="7" t="n"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>жомарт, береген, сараң емес адамды сипаттайды. Яғни адамның қолынан келгенінше көмектесетін, сый-сияпат жасауға дайын жомарт мінезін білдіреді.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J10" s="7" t="n"/>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="7" t="n"/>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>жомарт, мырза, қолында барын басқалардан аямайтын, қайырымды адамды білдіреді.</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M10" s="7" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1">
@@ -1584,14 +1754,36 @@
           <t>қатты ұялды</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="7" t="n"/>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>қатты ұялды, ұялғаннан беті қызарды деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G11" s="7" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="6" t="n"/>
-      <c r="L11" s="7" t="n"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>адамның қатты ұялғанын, қызарып кеткенін, ұятқа қалғанын білдіреді. Кейде қатты ызаланған, ашуланған күйін де сипаттайды.</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>қатты ұялуды, қысылуды немесе ыңғайсыз жағдайда қалып, беті дуылдап қызаруды білдіреді.</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M11" s="7" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1">
@@ -1613,14 +1805,32 @@
           <t>өте тату</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="7" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>өте тату, бір-біріне жақын деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G12" s="7" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="7" t="n"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>екі адамның өте жақын, тығыз қарым-қатынаста екенін, араларына ешкімнің кіріге алмайтынын білдіреді. Сондай-ақ бір нәрсенің тығыз, мызғымас, берік екенін сипаттауда да қолданылады.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J12" s="7" t="n"/>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="7" t="n"/>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>екі адамның арасындағы өте тығыз достықты, айырылмас татулықты, сыйластық пен бірлікті білдіреді.</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M12" s="7" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1">
@@ -1642,14 +1852,32 @@
           <t>момын, жуас</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="7" t="n"/>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>өте жуас, момын, ешкімге зияны жоқ деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G13" s="7" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="7" t="n"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>өте момын, жуас, жұмсақ мінезді, ешкімге зияны жоқ адамды сипаттайды. Яғни адамның ұрыспайтын, ашуланбайтын, мүлдем зиянсыз, көнбіс мінезін білдіреді.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J13" s="7" t="n"/>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="7" t="n"/>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>өте момын, жуас, ешкімге залалы тимейтін, тыныш әрі бейуаз адамды білдіреді.</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M13" s="7" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1">
@@ -1671,14 +1899,32 @@
           <t>лық толы, бос орын жоқ</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="7" t="n"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>адам өте көп, бос орын жоқ деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G14" s="7" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="7" t="n"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>адамның өте тығыз, лық толы, көпшілік қаумалаған жағдайын білдіреді. Яғни айналада бос орын жоқ, адамдар тым көп деген мағынаны білдіреді.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J14" s="7" t="n"/>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="7" t="n"/>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>орынның өте лық толы екенін, бос жер мүлдем жоқ екенін немесе халықтың шектен тыс көп жиналғанын білдіреді.</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M14" s="7" t="n"/>
     </row>
     <row r="15" ht="45" customHeight="1">
@@ -1700,14 +1946,32 @@
           <t>өте қиын, ауыр, ұзақ іс</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="7" t="n"/>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>көп еңбекті, шыдамдылық пен табандылықты қажет ететін қиын істі білдіретін тұрақты тіркес.</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G15" s="7" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="7" t="n"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Ол өте ауыр, азапты, ұзақ әрі нәтижесіз немесе асқан шыдамдылықты қажет ететін жұмыс деген мағынаны білдіреді</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J15" s="7" t="n"/>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="7" t="n"/>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>өте үлкен сабырды, төзімділікті, ұқыптылықты және қажырлы еңбекті талап ететін аса қиын әрі баяу жүретін істі сипаттайтын бейнелі тіркес</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M15" s="7" t="n"/>
     </row>
     <row r="16" ht="45" customHeight="1">
@@ -1729,14 +1993,32 @@
           <t>қатты ұялу</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="7" t="n"/>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>қатты ұялу, қысылу, ұялғаннан тығылар жер таппау деген мағынаны білдіретін тұрақты тіркес.</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G16" s="7" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="7" t="n"/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>қатты ұялып, не істерін білмей қалу, «жерге кіріп кетердей болу» дегенді білдіреді</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J16" s="7" t="n"/>
-      <c r="K16" s="6" t="n"/>
-      <c r="L16" s="7" t="n"/>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>қатты ұялғаннан, айыпты болғаннан немесе ыңғайсыз жағдайға тап болғаннан жасырынатын жер таппай, не істерін білмей сасқалақтауды білдіретін тұрақты тіркес.</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" s="7" t="n"/>
     </row>
     <row r="17" ht="45" customHeight="1">
@@ -1758,14 +2040,32 @@
           <t>тар, кішкентай жер</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="7" t="n"/>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>көлемі өте кішкентай, шағын деген мағына</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G17" s="7" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="7" t="n"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>«өте шағын, тар, кішкентай» дегенді білдіреді</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J17" s="7" t="n"/>
-      <c r="K17" s="6" t="n"/>
-      <c r="L17" s="7" t="n"/>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>аумағы немесе көлемі өте шағын, кішкентай, тұтастай көзге сиып тұратын жерді, орынды немесе затты сипаттайтын тұрақты тіркес.</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M17" s="7" t="n"/>
     </row>
     <row r="18" ht="45" customHeight="1">
@@ -1787,14 +2087,32 @@
           <t>тып-тыныш</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="7" t="n"/>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>тым-тырыс, ешбір дыбыс естілмейтін тыныштық</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G18" s="7" t="n"/>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="7" t="n"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>«тып-тыныш, жым-жырт», яғни айналада ешбір дыбыс естілмейтін, мүлдем тыныштық орнаған күйді білдіреді</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J18" s="7" t="n"/>
-      <c r="K18" s="6" t="n"/>
-      <c r="L18" s="7" t="n"/>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>айналада ешқандай дыбыс, дабыра жоқ, айналаның жым-жырт, тып-тыныш болып мүлгіп тұрған күйін білдіретін тұрақты тіркес.</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M18" s="7" t="n"/>
     </row>
     <row r="19" ht="45" customHeight="1">
@@ -1816,14 +2134,32 @@
           <t>үндемейтін адам</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="7" t="n"/>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>үндемей, ештеңе айтпай отыру</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G19" s="7" t="n"/>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="7" t="n"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>«үндемейтін адам, ауыз ашпайтын, сөйлемейтін адам»</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J19" s="7" t="n"/>
-      <c r="K19" s="6" t="n"/>
-      <c r="L19" s="7" t="n"/>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>ештеңе айтпай, мүлдем сөйлемей, сұрақтарға жауап бермей ләм-мим демей отырып алу</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M19" s="7" t="n"/>
     </row>
     <row r="20" ht="45" customHeight="1">
@@ -1845,14 +2181,32 @@
           <t>батыр, қорықпайтын</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="7" t="n"/>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>өте батыл, ержүрек, ештеңеден қорықпайтын адам</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G20" s="7" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="7" t="n"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>«батыр, ержүрек, ешнәрседен қорықпайтын адам»</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J20" s="7" t="n"/>
-      <c r="K20" s="6" t="n"/>
-      <c r="L20" s="7" t="n"/>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>ештеңеден қорықпайтын, қауіп-қатерге қаймықпай қарсы тұратын, өте батыл, өжет әрі қайсар адам</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M20" s="7" t="n"/>
     </row>
     <row r="21" ht="45" customHeight="1">
@@ -1874,14 +2228,32 @@
           <t>қу, айлакер</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="7" t="n"/>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>болмашы нәрседен де пайда табуға тырысатын, айлакер, қу адам</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G21" s="7" t="n"/>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="7" t="n"/>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>«тым сараң, қу, пайдакүнем»</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J21" s="7" t="n"/>
-      <c r="K21" s="6" t="n"/>
-      <c r="L21" s="7" t="n"/>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>өте сараң, тым есепшіл, ешқандай мүмкіндік жоқ жерден де пайда тапқысы келетін шектен шыққан дүниеқоңыз, ашқарақ адам</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M21" s="7" t="n"/>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -1903,14 +2275,32 @@
           <t>хан сайлады</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="7" t="n"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>хан сайлады</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G22" s="7" t="n"/>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="7" t="n"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>хан көтерді, таққа отырғызды</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J22" s="7" t="n"/>
-      <c r="K22" s="6" t="n"/>
-      <c r="L22" s="7" t="n"/>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>хан етіп сайлады, ел басшысы етіп ұлықтады немесе бір адамға ерекше құрмет көрсетіп, жоғары дәрежеге көтерді</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M22" s="7" t="n"/>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -1932,14 +2322,32 @@
           <t>жолы болды</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="7" t="n"/>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>жолы болды, ісі оңға басты, сәттілікке жетті</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G23" s="7" t="n"/>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="7" t="n"/>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>ісі оңға басты, сәті түсті, жолы болды</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J23" s="7" t="n"/>
-      <c r="K23" s="6" t="n"/>
-      <c r="L23" s="7" t="n"/>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>ісі оңға басып, бағы жанды, жолы болып, сәттілікке кенелді</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M23" s="7" t="n"/>
     </row>
     <row r="24" ht="45" customHeight="1">
@@ -1961,14 +2369,32 @@
           <t>молшылық орнау</t>
         </is>
       </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="7" t="n"/>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>молшылыққа кенелу, ішіп-жемнің ағыл-тегіл көп болуы</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G24" s="7" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="7" t="n"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>молшылық, береке, тоқшылық орнау</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J24" s="7" t="n"/>
-      <c r="K24" s="6" t="n"/>
-      <c r="L24" s="7" t="n"/>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>тұрмыс-тіршілікте азық-түлік, мал-жан, ақ (сүт өнімдері) өте мол болып, шалқыған тоқшылық пен береке орнаған кез</t>
+        </is>
+      </c>
+      <c r="L24" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M24" s="7" t="n"/>
     </row>
     <row r="25" ht="45" customHeight="1">
@@ -1990,14 +2416,32 @@
           <t>тыныш, бейбіт заман орнау</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="7" t="n"/>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>елде тыныштық, бейбітшілік пен молшылық орнау</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G25" s="7" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="7" t="n"/>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>бейбіт, тыныш, молшылық заман орнау</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J25" s="7" t="n"/>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="7" t="n"/>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>елде толық тыныштық пен бейбітшілік орнаған, ешқандай қауіп-қатерсіз, мамыражай, берекелі де тоқ заман</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M25" s="7" t="n"/>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -2019,15 +2463,37 @@
           <t>баю</t>
         </is>
       </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="7" t="n"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>баю, шалқып, молшылықта өмір сүру</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G26" s="7" t="n"/>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="7" t="n"/>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>баю, дәулеті асу, байып кету</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J26" s="7" t="n"/>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="7" t="n"/>
-      <c r="M26" s="7" t="n"/>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>аяқастынан ашуға міну, шамдану, мінез көрсетіп, тулап шыға келу</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>О</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="4" t="n">
@@ -2048,14 +2514,32 @@
           <t>қатты ұрысу, балағаттау</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="7" t="n"/>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>қатты ұрысу, балағаттау, жер-жебіріне жету</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G27" s="7" t="n"/>
-      <c r="H27" s="6" t="n"/>
-      <c r="I27" s="7" t="n"/>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>қатты ұрысу, балағаттау, сөгу</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J27" s="7" t="n"/>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="7" t="n"/>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>бір адамды аямай қатты ұрсу, жер-жебіріне жету, ауыр сөздер айтып, жерден алып жерге салу</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M27" s="7" t="n"/>
     </row>
     <row r="28" ht="45" customHeight="1">
@@ -2077,15 +2561,41 @@
           <t>алдау</t>
         </is>
       </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="7" t="n"/>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>жеңу, жеңіліске ұшырату</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>О</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>алдау, алаяқтық жасау</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J28" s="7" t="n"/>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="7" t="n"/>
-      <c r="M28" s="7" t="n"/>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>біреуді ойсырата жеңу, айласын асырып сүріндіру немесе тиісті сазайын беріп, сағын сындыру</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
+        <is>
+          <t>О</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="4" t="n">
@@ -2106,14 +2616,32 @@
           <t>өте алыс жер</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="7" t="n"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>өте алыс, шалғай жер</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G29" s="7" t="n"/>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="7" t="n"/>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>тым алыс, қашық, қияндағы жер</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J29" s="7" t="n"/>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="7" t="n"/>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>өте алыстағы, жетуі қиын, шеткері, адам аяғы сирек басатын немесе елсіз, қаңырап қалған шалғай аймақ</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M29" s="7" t="n"/>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -2135,14 +2663,36 @@
           <t>асқақтап, дәурен сүру</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="7" t="n"/>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>жолы болып, бағы жану, дәурені жүру</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G30" s="7" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="7" t="n"/>
-      <c r="J30" s="7" t="n"/>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="7" t="n"/>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>мақтанып, тәкаппарлану, өзін жоғары санау</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>О</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>бағы жанып, ісі оңға басып, абыройы мен мерейі тасып, өркендеп тұрған немесе еңсесі көтеріңкі күй</t>
+        </is>
+      </c>
+      <c r="L30" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M30" s="7" t="n"/>
     </row>
     <row r="31" ht="45" customHeight="1">
@@ -2164,14 +2714,32 @@
           <t>масқаралау, ел алдында ұятқа қалдыру</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="7" t="n"/>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>ел алдында масқаралау, мазақ ету, абыройын төгу</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G31" s="7" t="n"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="7" t="n"/>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>артына кір келтіру, ұятқа қалдыру, масқаралау</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J31" s="7" t="n"/>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="7" t="n"/>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>біреудің абыройын айрандай төгіп, ел алдында масқаралау, қатты жазалау немесе беделін жұрт алдында мүлдем түсіру</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M31" s="7" t="n"/>
     </row>
   </sheetData>
@@ -2298,14 +2866,32 @@
           <t>Беті бүлк етпеді (ұялды – ұялмады)</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="7" t="n"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>«Беті бүлк етпеді» — ұялмады, қысылмады</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G2" s="7" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="7" t="n"/>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>беті бүлк етпеді</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J2" s="7" t="n"/>
-      <c r="K2" s="6" t="n"/>
-      <c r="L2" s="7" t="n"/>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Беті бүлк етпеу</t>
+        </is>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M2" s="7" t="n"/>
     </row>
     <row r="3" ht="40" customHeight="1">
@@ -2327,15 +2913,41 @@
           <t>Қуанышы қойнына сыймады (мұңайды – қуанды)</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="7" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="7" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>«Ажары кірді» — өңі жақсарды, көріктене түсті</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>«қуанышы қойнына сыймады» (қуаныштан іші-бауыры қызу, қатты қуану) тіркесі</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J3" s="7" t="n"/>
-      <c r="K3" s="6" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="7" t="n"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Жүзіне қан жүгіру</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="4" t="n">
@@ -2356,14 +2968,32 @@
           <t>Саусағының ұшын қимылдатпады (тез қимылдады – ештеңе істемеді)</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="7" t="n"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>«Қол қусырып отырды» — ештеңе істемеді, әрекетсіз отырды</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G4" s="7" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="7" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Саусағының ұшын қимылдатпады</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J4" s="7" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="7" t="n"/>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Саусағының ұшын да қимылдатпау</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M4" s="7" t="n"/>
     </row>
     <row r="5" ht="40" customHeight="1">
@@ -2385,14 +3015,36 @@
           <t>Қыздың жиған жүгіндей (сұлу, әдемі)</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="7" t="n"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>«Ай десе аузы, күн десе көзі бар» — өте сұлу, көрікті</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Қыздың жиған жүгіндей</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J5" s="7" t="n"/>
-      <c r="K5" s="6" t="n"/>
-      <c r="L5" s="7" t="n"/>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Сұлулығына көз сүрінеді</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M5" s="7" t="n"/>
     </row>
     <row r="6" ht="40" customHeight="1">
@@ -2414,14 +3066,32 @@
           <t>Ит арқасы қиянда; Жер түбі (алыс, шалғай)</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>«Ит арқасы қиянда» — өте алыс, шалғайда</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G6" s="7" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="7" t="n"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Ит арқасы қиян</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="7" t="n"/>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Ит арқасы қиянда</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M6" s="7" t="n"/>
     </row>
     <row r="7" ht="40" customHeight="1">
@@ -2443,14 +3113,33 @@
           <t>Жерден алып, жерге салды (ұрысты, сөкті)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>«Жер-жебіріне жетті» — қатты ұрысты,</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G7" s="7" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="7" t="n"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>«жерден алып, жерге салды» — ұрысты, сөкті</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="J7" s="7" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="7" t="n"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Жер-жебіріне жету
+Жерден алып, жерге салу</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="M7" s="7" t="n"/>
     </row>
     <row r="9">
@@ -2544,11 +3233,23 @@
       <c r="B2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="n"/>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Көзді ашып-жұмғанша</t>
+        </is>
+      </c>
       <c r="D2" s="7" t="n"/>
-      <c r="E2" s="6" t="n"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Көзді ашып-жұмғанша</t>
+        </is>
+      </c>
       <c r="F2" s="7" t="n"/>
-      <c r="G2" s="6" t="n"/>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Көзді ашып-жұмғанша</t>
+        </is>
+      </c>
       <c r="H2" s="7" t="n"/>
     </row>
     <row r="3">
@@ -2556,11 +3257,23 @@
       <c r="B3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="n"/>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Қас пен көздің арасында</t>
+        </is>
+      </c>
       <c r="D3" s="7" t="n"/>
-      <c r="E3" s="6" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Қас пен көздің арасында</t>
+        </is>
+      </c>
       <c r="F3" s="7" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Қас пен көздің арасында</t>
+        </is>
+      </c>
       <c r="H3" s="7" t="n"/>
     </row>
     <row r="4">
@@ -2568,11 +3281,23 @@
       <c r="B4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="6" t="n"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Кірпік қаққанша</t>
+        </is>
+      </c>
       <c r="D4" s="7" t="n"/>
-      <c r="E4" s="6" t="n"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Аяғы аяғына жұқпады</t>
+        </is>
+      </c>
       <c r="F4" s="7" t="n"/>
-      <c r="G4" s="6" t="n"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Аяғы аяғына тимеу</t>
+        </is>
+      </c>
       <c r="H4" s="7" t="n"/>
     </row>
     <row r="5">
@@ -2580,11 +3305,27 @@
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="6" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Әп дегенше</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Қас қағымда</t>
+        </is>
+      </c>
       <c r="F5" s="7" t="n"/>
-      <c r="G5" s="6" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Оқтай атылу</t>
+        </is>
+      </c>
       <c r="H5" s="7" t="n"/>
     </row>
     <row r="6">
@@ -2592,11 +3333,23 @@
       <c r="B6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="6" t="n"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Аяқ-аяғына жұқпау</t>
+        </is>
+      </c>
       <c r="D6" s="7" t="n"/>
-      <c r="E6" s="6" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Ерні ерніне тимеді</t>
+        </is>
+      </c>
       <c r="F6" s="7" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Желдей есу</t>
+        </is>
+      </c>
       <c r="H6" s="7" t="n"/>
     </row>
     <row r="7">
@@ -2608,11 +3361,23 @@
       <c r="B7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="6" t="n"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Ит өлген жер</t>
+        </is>
+      </c>
       <c r="D7" s="7" t="n"/>
-      <c r="E7" s="6" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Ит өлген жер</t>
+        </is>
+      </c>
       <c r="F7" s="7" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Ит өлген жер</t>
+        </is>
+      </c>
       <c r="H7" s="7" t="n"/>
     </row>
     <row r="8">
@@ -2620,11 +3385,23 @@
       <c r="B8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Ит арқасы қиянда</t>
+        </is>
+      </c>
       <c r="D8" s="7" t="n"/>
-      <c r="E8" s="6" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Ит арқасы қиянда</t>
+        </is>
+      </c>
       <c r="F8" s="7" t="n"/>
-      <c r="G8" s="6" t="n"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Ит арқасы қиянда</t>
+        </is>
+      </c>
       <c r="H8" s="7" t="n"/>
     </row>
     <row r="9">
@@ -2632,11 +3409,23 @@
       <c r="B9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="6" t="n"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Жердің түбі</t>
+        </is>
+      </c>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="6" t="n"/>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Қиянның қиынында</t>
+        </is>
+      </c>
       <c r="F9" s="7" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Жердің түбінде</t>
+        </is>
+      </c>
       <c r="H9" s="7" t="n"/>
     </row>
     <row r="10">
@@ -2644,11 +3433,23 @@
       <c r="B10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="6" t="n"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Жер мойны қашық</t>
+        </is>
+      </c>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="6" t="n"/>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Ат тұяғы тимеген</t>
+        </is>
+      </c>
       <c r="F10" s="7" t="n"/>
-      <c r="G10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Ат табаны жетпейтін жер</t>
+        </is>
+      </c>
       <c r="H10" s="7" t="n"/>
     </row>
     <row r="11">
@@ -2656,12 +3457,32 @@
       <c r="B11" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="6" t="n"/>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Айшылық алыс жер</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Қиыр шет</t>
+        </is>
+      </c>
       <c r="F11" s="7" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="7" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Айшылық жер</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -2672,11 +3493,23 @@
       <c r="B12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="6" t="n"/>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Таяқ тастам жер</t>
+        </is>
+      </c>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="6" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>қол созым жер</t>
+        </is>
+      </c>
       <c r="F12" s="7" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Таяқ тастам жер</t>
+        </is>
+      </c>
       <c r="H12" s="7" t="n"/>
     </row>
     <row r="13">
@@ -2684,11 +3517,23 @@
       <c r="B13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="6" t="n"/>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Қарға адым жер</t>
+        </is>
+      </c>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="6" t="n"/>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>көз жететін жер</t>
+        </is>
+      </c>
       <c r="F13" s="7" t="n"/>
-      <c r="G13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Қол созым жер</t>
+        </is>
+      </c>
       <c r="H13" s="7" t="n"/>
     </row>
     <row r="14">
@@ -2696,11 +3541,27 @@
       <c r="B14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="6" t="n"/>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Қол созым жер</t>
+        </is>
+      </c>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>үш қайнаса сорпасы қосылмайтын</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Екі адым жер</t>
+        </is>
+      </c>
       <c r="H14" s="7" t="n"/>
     </row>
     <row r="15">
@@ -2708,23 +3569,59 @@
       <c r="B15" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="7" t="n"/>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Иек астында</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>ат құлағында ойнайтын</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Мұрын түбінде (немесе Мұрын астында)</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
       <c r="B16" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="7" t="n"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Тиіп тұр</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="7" t="n"/>
-      <c r="G16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Ат аттам жер</t>
+        </is>
+      </c>
       <c r="H16" s="7" t="n"/>
     </row>
     <row r="17">
@@ -2736,11 +3633,23 @@
       <c r="B17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="6" t="n"/>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Құмырсқадай құжынаған</t>
+        </is>
+      </c>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="6" t="n"/>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Қарасы қалың</t>
+        </is>
+      </c>
       <c r="F17" s="7" t="n"/>
-      <c r="G17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Ине шаншар жер жоқ</t>
+        </is>
+      </c>
       <c r="H17" s="7" t="n"/>
     </row>
     <row r="18">
@@ -2748,23 +3657,51 @@
       <c r="B18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C18" s="6" t="n"/>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Қара құрым</t>
+        </is>
+      </c>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="6" t="n"/>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Қалың қол</t>
+        </is>
+      </c>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="7" t="n"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Қара ормандай</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n"/>
       <c r="B19" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="6" t="n"/>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Ине шаншар жер жоқ</t>
+        </is>
+      </c>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="6" t="n"/>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Қалың бұқара</t>
+        </is>
+      </c>
       <c r="F19" s="7" t="n"/>
-      <c r="G19" s="6" t="n"/>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Құмырсқадай өру</t>
+        </is>
+      </c>
       <c r="H19" s="7" t="n"/>
     </row>
     <row r="20">
@@ -2772,11 +3709,31 @@
       <c r="B20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="6" t="n"/>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Құмдай көп</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Бір кісідей бар екен</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Иін тіресу</t>
+        </is>
+      </c>
       <c r="H20" s="7" t="n"/>
     </row>
     <row r="21">
@@ -2784,11 +3741,27 @@
       <c r="B21" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C21" s="6" t="n"/>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Жер қайысқан қол</t>
+        </is>
+      </c>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="6" t="n"/>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Ел-жұрттың қарасы қалың</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Қара құрттай қаптау</t>
+        </is>
+      </c>
       <c r="H21" s="7" t="n"/>
     </row>
     <row r="22">
@@ -2800,11 +3773,23 @@
       <c r="B22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="6" t="n"/>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Қас қарая</t>
+        </is>
+      </c>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="6" t="n"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Қас қарайды</t>
+        </is>
+      </c>
       <c r="F22" s="7" t="n"/>
-      <c r="G22" s="6" t="n"/>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Қас қарайғанда</t>
+        </is>
+      </c>
       <c r="H22" s="7" t="n"/>
     </row>
     <row r="23">
@@ -2812,11 +3797,27 @@
       <c r="B23" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C23" s="6" t="n"/>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Көз байлана</t>
+        </is>
+      </c>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="6" t="n"/>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Күн батты</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Көз байланғанда</t>
+        </is>
+      </c>
       <c r="H23" s="7" t="n"/>
     </row>
     <row r="24">
@@ -2824,11 +3825,23 @@
       <c r="B24" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C24" s="6" t="n"/>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Екі кештің арасында</t>
+        </is>
+      </c>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="6" t="n"/>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Ымырт үйірілді</t>
+        </is>
+      </c>
       <c r="F24" s="7" t="n"/>
-      <c r="G24" s="6" t="n"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Ел орынға отыра</t>
+        </is>
+      </c>
       <c r="H24" s="7" t="n"/>
     </row>
     <row r="25">
@@ -2836,11 +3849,23 @@
       <c r="B25" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C25" s="6" t="n"/>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Ел орынға отыра</t>
+        </is>
+      </c>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="6" t="n"/>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Ақшам түсті</t>
+        </is>
+      </c>
       <c r="F25" s="7" t="n"/>
-      <c r="G25" s="6" t="n"/>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Алакеуім шақта</t>
+        </is>
+      </c>
       <c r="H25" s="7" t="n"/>
     </row>
     <row r="26">
@@ -2848,11 +3873,27 @@
       <c r="B26" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C26" s="6" t="n"/>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Күн ұясына кіргенде</t>
+        </is>
+      </c>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="6" t="n"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Түн ортасы</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Т</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Ақшам түсе</t>
+        </is>
+      </c>
       <c r="H26" s="7" t="n"/>
     </row>
   </sheetData>
@@ -2902,7 +3943,11 @@
           <t>ЖИ-1</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n"/>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2910,7 +3955,11 @@
           <t>ЖИ-2</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n"/>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2918,7 +3967,11 @@
           <t>ЖИ-3</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">

</xml_diff>